<commit_message>
atualizacao de 2 documentos
</commit_message>
<xml_diff>
--- a/Milestone 3/Plano de Projeto/Cronograma.xlsx
+++ b/Milestone 3/Plano de Projeto/Cronograma.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29328"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guiba\Desktop\LDS\Plano de Projeto\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utilizador\OneDrive\Documentos\GitHub\LDS\Milestone 3\Plano de Projeto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B71CF8BA-BD01-4B8E-B7C7-587C9230BB28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C99E1E5D-E6F9-4BAC-A307-BF1F5CBD85FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13152" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GanttChart" sheetId="9" r:id="rId1"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">GanttChart!$B$1:$BN$39</definedName>
     <definedName name="prevWBS" localSheetId="0">GanttChart!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">GanttChart!$B$1:$BN$37</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">GanttChart!$4:$7</definedName>
     <definedName name="valuevx">42.314159</definedName>
     <definedName name="vertex42_copyright" hidden="1">"© 2006-2018 Vertex42 LLC"</definedName>
@@ -38,45 +38,8 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>Vertex42</author>
-  </authors>
-  <commentList>
-    <comment ref="D7" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000004000000}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Predecessor Tasks:
-</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>You can use this column to enter the WBS of a predecessor for reference. The PRO version uses formulas to automatically calculate the Start Date based on the Predecessor.</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="44">
-  <si>
-    <t>PREDECESSOR</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="46">
   <si>
     <t xml:space="preserve">Consulta+ </t>
   </si>
@@ -206,6 +169,15 @@
   <si>
     <t>PipeLine funcional com testesno BE</t>
   </si>
+  <si>
+    <t>Trabalho ES2</t>
+  </si>
+  <si>
+    <t>Trabalho ED</t>
+  </si>
+  <si>
+    <t>Diogo, Guilherme, André</t>
+  </si>
 </sst>
 </file>
 
@@ -217,7 +189,7 @@
     <numFmt numFmtId="166" formatCode="d\ mmm\ yyyy"/>
     <numFmt numFmtId="167" formatCode="[$-816]d/mmm;@"/>
   </numFmts>
-  <fonts count="40" x14ac:knownFonts="1">
+  <fonts count="37" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -380,19 +352,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="9"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -445,13 +404,6 @@
     <font>
       <b/>
       <sz val="9"/>
-      <name val="Arial"/>
-      <family val="2"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="major"/>
@@ -942,24 +894,24 @@
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="32" fillId="22" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="30" fillId="22" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="32" fillId="22" borderId="11" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="9" fontId="30" fillId="22" borderId="11" xfId="40" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="32" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="30" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -971,48 +923,45 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="1" fontId="34" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="32" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="28" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="26" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -1027,13 +976,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="23" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="28" fillId="23" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="23" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="32" fillId="21" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="30" fillId="21" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="32" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="30" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1045,87 +994,90 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="34" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="34" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="29" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="29" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="29" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="34" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="34" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="164" fontId="31" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="29" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="31" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="167" fontId="29" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="166" fontId="31" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="31" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="44">
-    <cellStyle name="20% - Accent1" xfId="1" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Accent2" xfId="2" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Accent3" xfId="3" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Accent4" xfId="4" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Accent5" xfId="5" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Accent6" xfId="6" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Accent1" xfId="7" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Accent2" xfId="8" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Accent3" xfId="9" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Accent4" xfId="10" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Accent5" xfId="11" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Accent6" xfId="12" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Accent1" xfId="13" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Accent2" xfId="14" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Accent3" xfId="15" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Accent4" xfId="16" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Accent5" xfId="17" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Accent6" xfId="18" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Accent1" xfId="19" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Accent2" xfId="20" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Accent3" xfId="21" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Accent4" xfId="22" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Accent5" xfId="23" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Accent6" xfId="24" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Bad" xfId="25" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Calculation" xfId="26" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Check Cell" xfId="27" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Explanatory Text" xfId="28" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Good" xfId="29" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Heading 1" xfId="30" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Heading 2" xfId="31" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Heading 3" xfId="32" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Heading 4" xfId="33" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Hyperlink" xfId="34" builtinId="8"/>
-    <cellStyle name="Input" xfId="35" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Linked Cell" xfId="36" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Neutral" xfId="37" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="20% - Cor1" xfId="1" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - Cor2" xfId="2" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - Cor3" xfId="3" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - Cor4" xfId="4" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - Cor5" xfId="5" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - Cor6" xfId="6" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - Cor1" xfId="7" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - Cor2" xfId="8" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - Cor3" xfId="9" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - Cor4" xfId="10" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - Cor5" xfId="11" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - Cor6" xfId="12" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - Cor1" xfId="13" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - Cor2" xfId="14" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - Cor3" xfId="15" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - Cor4" xfId="16" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - Cor5" xfId="17" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - Cor6" xfId="18" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="Cabeçalho 1" xfId="30" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="Cabeçalho 2" xfId="31" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="Cabeçalho 3" xfId="32" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="Cabeçalho 4" xfId="33" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="Cálculo" xfId="26" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="Célula Ligada" xfId="36" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="Cor1" xfId="19" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="Cor2" xfId="20" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="Cor3" xfId="21" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="Cor4" xfId="22" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="Cor5" xfId="23" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="Cor6" xfId="24" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="Correto" xfId="29" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="Entrada" xfId="35" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="Hiperligação" xfId="34" builtinId="8"/>
+    <cellStyle name="Incorreto" xfId="25" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="Neutro" xfId="37" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Note" xfId="38" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Output" xfId="39" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Percent" xfId="40" builtinId="5"/>
-    <cellStyle name="Title" xfId="41" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="Nota" xfId="38" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="Percentagem" xfId="40" builtinId="5"/>
+    <cellStyle name="Saída" xfId="39" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="Texto de Aviso" xfId="43" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Texto Explicativo" xfId="28" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="Título" xfId="41" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Total" xfId="42" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="Warning Text" xfId="43" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="Verificar Célula" xfId="27" builtinId="23" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
@@ -1259,16 +1211,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="absolute">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>373959</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>427299</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>69160</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>118533</xdr:rowOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>57730</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>8043</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1323,11 +1275,11 @@
           <xdr:col>9</xdr:col>
           <xdr:colOff>95250</xdr:colOff>
           <xdr:row>1</xdr:row>
-          <xdr:rowOff>123825</xdr:rowOff>
+          <xdr:rowOff>125730</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>27</xdr:col>
-          <xdr:colOff>104775</xdr:colOff>
+          <xdr:colOff>106680</xdr:colOff>
           <xdr:row>2</xdr:row>
           <xdr:rowOff>114300</xdr:rowOff>
         </xdr:to>
@@ -1659,65 +1611,65 @@
   <sheetPr codeName="Sheet8">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BN37"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:BN39"/>
+  <sheetFormatPr defaultColWidth="9.1640625" defaultRowHeight="12.3" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="6.140625" style="34" customWidth="1"/>
-    <col min="2" max="2" width="30.5703125" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" customWidth="1"/>
-    <col min="4" max="4" width="8.140625" hidden="1" customWidth="1"/>
-    <col min="5" max="6" width="10.7109375" customWidth="1"/>
+    <col min="1" max="1" width="6.1640625" style="33" customWidth="1"/>
+    <col min="2" max="2" width="30.5546875" customWidth="1"/>
+    <col min="3" max="3" width="10.71875" customWidth="1"/>
+    <col min="4" max="4" width="9.94140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10.71875" customWidth="1"/>
     <col min="7" max="7" width="6" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="14.140625" customWidth="1"/>
-    <col min="10" max="10" width="1.85546875" customWidth="1"/>
-    <col min="11" max="66" width="2.42578125" customWidth="1"/>
+    <col min="9" max="9" width="14.1640625" customWidth="1"/>
+    <col min="10" max="10" width="1.83203125" customWidth="1"/>
+    <col min="11" max="66" width="2.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:66" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="27" t="s">
-        <v>1</v>
+    <row r="1" spans="1:66" ht="30" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="B1" s="26" t="s">
+        <v>0</v>
       </c>
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
       <c r="E1" s="5"/>
       <c r="F1" s="5"/>
-      <c r="I1" s="31"/>
-      <c r="K1" s="44" t="s">
-        <v>35</v>
-      </c>
-      <c r="L1" s="44"/>
-      <c r="M1" s="44"/>
-      <c r="N1" s="44"/>
-      <c r="O1" s="44"/>
-      <c r="P1" s="44"/>
-      <c r="Q1" s="44"/>
-      <c r="R1" s="44"/>
-      <c r="S1" s="44"/>
-      <c r="T1" s="44"/>
-      <c r="U1" s="44"/>
-      <c r="V1" s="44"/>
-      <c r="W1" s="44"/>
-      <c r="X1" s="44"/>
-      <c r="Y1" s="44"/>
-      <c r="Z1" s="44"/>
-      <c r="AA1" s="44"/>
-      <c r="AB1" s="44"/>
-      <c r="AC1" s="42"/>
-      <c r="AD1" s="42"/>
-      <c r="AE1" s="42"/>
+      <c r="I1" s="30"/>
+      <c r="K1" s="49" t="s">
+        <v>34</v>
+      </c>
+      <c r="L1" s="49"/>
+      <c r="M1" s="49"/>
+      <c r="N1" s="49"/>
+      <c r="O1" s="49"/>
+      <c r="P1" s="49"/>
+      <c r="Q1" s="49"/>
+      <c r="R1" s="49"/>
+      <c r="S1" s="49"/>
+      <c r="T1" s="49"/>
+      <c r="U1" s="49"/>
+      <c r="V1" s="49"/>
+      <c r="W1" s="49"/>
+      <c r="X1" s="49"/>
+      <c r="Y1" s="49"/>
+      <c r="Z1" s="49"/>
+      <c r="AA1" s="49"/>
+      <c r="AB1" s="49"/>
+      <c r="AC1" s="41"/>
+      <c r="AD1" s="41"/>
+      <c r="AE1" s="41"/>
     </row>
-    <row r="2" spans="1:66" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:66" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B2" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" s="33"/>
+        <v>1</v>
+      </c>
+      <c r="C2" s="32"/>
       <c r="D2" s="4"/>
-      <c r="E2" s="32"/>
-      <c r="F2" s="32"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
       <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:66" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:66" x14ac:dyDescent="0.4">
       <c r="B3" s="2"/>
       <c r="H3" s="1"/>
       <c r="K3" s="3"/>
@@ -1738,197 +1690,197 @@
       <c r="Z3" s="3"/>
       <c r="AA3" s="3"/>
     </row>
-    <row r="4" spans="1:66" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:66" ht="17.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B4" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="49">
+        <v>2</v>
+      </c>
+      <c r="C4" s="51">
         <v>45915</v>
       </c>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="43" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="43"/>
-      <c r="H4" s="30">
+      <c r="D4" s="51"/>
+      <c r="E4" s="51"/>
+      <c r="F4" s="48" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="48"/>
+      <c r="H4" s="29">
         <v>6</v>
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="6"/>
-      <c r="K4" s="46" t="str">
+      <c r="K4" s="42" t="str">
         <f>"Semana "&amp;(K6-($C$4-WEEKDAY($C$4,1)+2))/7+1</f>
         <v>Semana 6</v>
       </c>
-      <c r="L4" s="47"/>
-      <c r="M4" s="47"/>
-      <c r="N4" s="47"/>
-      <c r="O4" s="47"/>
-      <c r="P4" s="47"/>
-      <c r="Q4" s="48"/>
-      <c r="R4" s="46" t="str">
+      <c r="L4" s="43"/>
+      <c r="M4" s="43"/>
+      <c r="N4" s="43"/>
+      <c r="O4" s="43"/>
+      <c r="P4" s="43"/>
+      <c r="Q4" s="44"/>
+      <c r="R4" s="42" t="str">
         <f>"Semana "&amp;(R6-($C$4-WEEKDAY($C$4,1)+2))/7+1</f>
         <v>Semana 7</v>
       </c>
-      <c r="S4" s="47"/>
-      <c r="T4" s="47"/>
-      <c r="U4" s="47"/>
-      <c r="V4" s="47"/>
-      <c r="W4" s="47"/>
-      <c r="X4" s="48"/>
-      <c r="Y4" s="46" t="str">
+      <c r="S4" s="43"/>
+      <c r="T4" s="43"/>
+      <c r="U4" s="43"/>
+      <c r="V4" s="43"/>
+      <c r="W4" s="43"/>
+      <c r="X4" s="44"/>
+      <c r="Y4" s="42" t="str">
         <f>"Semana "&amp;(Y6-($C$4-WEEKDAY($C$4,1)+2))/7+1</f>
         <v>Semana 8</v>
       </c>
-      <c r="Z4" s="47"/>
-      <c r="AA4" s="47"/>
-      <c r="AB4" s="47"/>
-      <c r="AC4" s="47"/>
-      <c r="AD4" s="47"/>
-      <c r="AE4" s="48"/>
-      <c r="AF4" s="46" t="str">
+      <c r="Z4" s="43"/>
+      <c r="AA4" s="43"/>
+      <c r="AB4" s="43"/>
+      <c r="AC4" s="43"/>
+      <c r="AD4" s="43"/>
+      <c r="AE4" s="44"/>
+      <c r="AF4" s="42" t="str">
         <f>"Semana "&amp;(AF6-($C$4-WEEKDAY($C$4,1)+2))/7+1</f>
         <v>Semana 9</v>
       </c>
-      <c r="AG4" s="47"/>
-      <c r="AH4" s="47"/>
-      <c r="AI4" s="47"/>
-      <c r="AJ4" s="47"/>
-      <c r="AK4" s="47"/>
-      <c r="AL4" s="48"/>
-      <c r="AM4" s="46" t="str">
+      <c r="AG4" s="43"/>
+      <c r="AH4" s="43"/>
+      <c r="AI4" s="43"/>
+      <c r="AJ4" s="43"/>
+      <c r="AK4" s="43"/>
+      <c r="AL4" s="44"/>
+      <c r="AM4" s="42" t="str">
         <f>"Semana "&amp;(AM6-($C$4-WEEKDAY($C$4,1)+2))/7+1</f>
         <v>Semana 10</v>
       </c>
-      <c r="AN4" s="47"/>
-      <c r="AO4" s="47"/>
-      <c r="AP4" s="47"/>
-      <c r="AQ4" s="47"/>
-      <c r="AR4" s="47"/>
-      <c r="AS4" s="48"/>
-      <c r="AT4" s="46" t="str">
+      <c r="AN4" s="43"/>
+      <c r="AO4" s="43"/>
+      <c r="AP4" s="43"/>
+      <c r="AQ4" s="43"/>
+      <c r="AR4" s="43"/>
+      <c r="AS4" s="44"/>
+      <c r="AT4" s="42" t="str">
         <f>"Semana "&amp;(AT6-($C$4-WEEKDAY($C$4,1)+2))/7+1</f>
         <v>Semana 11</v>
       </c>
-      <c r="AU4" s="47"/>
-      <c r="AV4" s="47"/>
-      <c r="AW4" s="47"/>
-      <c r="AX4" s="47"/>
-      <c r="AY4" s="47"/>
-      <c r="AZ4" s="48"/>
-      <c r="BA4" s="46" t="str">
+      <c r="AU4" s="43"/>
+      <c r="AV4" s="43"/>
+      <c r="AW4" s="43"/>
+      <c r="AX4" s="43"/>
+      <c r="AY4" s="43"/>
+      <c r="AZ4" s="44"/>
+      <c r="BA4" s="42" t="str">
         <f>"Semana "&amp;(BA6-($C$4-WEEKDAY($C$4,1)+2))/7+1</f>
         <v>Semana 12</v>
       </c>
-      <c r="BB4" s="47"/>
-      <c r="BC4" s="47"/>
-      <c r="BD4" s="47"/>
-      <c r="BE4" s="47"/>
-      <c r="BF4" s="47"/>
-      <c r="BG4" s="48"/>
-      <c r="BH4" s="46" t="str">
+      <c r="BB4" s="43"/>
+      <c r="BC4" s="43"/>
+      <c r="BD4" s="43"/>
+      <c r="BE4" s="43"/>
+      <c r="BF4" s="43"/>
+      <c r="BG4" s="44"/>
+      <c r="BH4" s="42" t="str">
         <f>"Semana "&amp;(BH6-($C$4-WEEKDAY($C$4,1)+2))/7+1</f>
         <v>Semana 13</v>
       </c>
-      <c r="BI4" s="47"/>
-      <c r="BJ4" s="47"/>
-      <c r="BK4" s="47"/>
-      <c r="BL4" s="47"/>
-      <c r="BM4" s="47"/>
-      <c r="BN4" s="48"/>
+      <c r="BI4" s="43"/>
+      <c r="BJ4" s="43"/>
+      <c r="BK4" s="43"/>
+      <c r="BL4" s="43"/>
+      <c r="BM4" s="43"/>
+      <c r="BN4" s="44"/>
     </row>
-    <row r="5" spans="1:66" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:66" ht="17.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B5" s="19"/>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
+      <c r="C5" s="50"/>
+      <c r="D5" s="50"/>
+      <c r="E5" s="50"/>
       <c r="F5" s="18"/>
       <c r="G5" s="18"/>
       <c r="H5" s="18"/>
       <c r="I5" s="18"/>
       <c r="J5" s="6"/>
-      <c r="K5" s="50">
+      <c r="K5" s="45">
         <f>K6</f>
         <v>45950</v>
       </c>
-      <c r="L5" s="51"/>
-      <c r="M5" s="51"/>
-      <c r="N5" s="51"/>
-      <c r="O5" s="51"/>
-      <c r="P5" s="51"/>
-      <c r="Q5" s="52"/>
-      <c r="R5" s="50">
+      <c r="L5" s="46"/>
+      <c r="M5" s="46"/>
+      <c r="N5" s="46"/>
+      <c r="O5" s="46"/>
+      <c r="P5" s="46"/>
+      <c r="Q5" s="47"/>
+      <c r="R5" s="45">
         <f>R6</f>
         <v>45957</v>
       </c>
-      <c r="S5" s="51"/>
-      <c r="T5" s="51"/>
-      <c r="U5" s="51"/>
-      <c r="V5" s="51"/>
-      <c r="W5" s="51"/>
-      <c r="X5" s="52"/>
-      <c r="Y5" s="50">
+      <c r="S5" s="46"/>
+      <c r="T5" s="46"/>
+      <c r="U5" s="46"/>
+      <c r="V5" s="46"/>
+      <c r="W5" s="46"/>
+      <c r="X5" s="47"/>
+      <c r="Y5" s="45">
         <f>Y6</f>
         <v>45964</v>
       </c>
-      <c r="Z5" s="51"/>
-      <c r="AA5" s="51"/>
-      <c r="AB5" s="51"/>
-      <c r="AC5" s="51"/>
-      <c r="AD5" s="51"/>
-      <c r="AE5" s="52"/>
-      <c r="AF5" s="50">
+      <c r="Z5" s="46"/>
+      <c r="AA5" s="46"/>
+      <c r="AB5" s="46"/>
+      <c r="AC5" s="46"/>
+      <c r="AD5" s="46"/>
+      <c r="AE5" s="47"/>
+      <c r="AF5" s="45">
         <f>AF6</f>
         <v>45971</v>
       </c>
-      <c r="AG5" s="51"/>
-      <c r="AH5" s="51"/>
-      <c r="AI5" s="51"/>
-      <c r="AJ5" s="51"/>
-      <c r="AK5" s="51"/>
-      <c r="AL5" s="52"/>
-      <c r="AM5" s="50">
+      <c r="AG5" s="46"/>
+      <c r="AH5" s="46"/>
+      <c r="AI5" s="46"/>
+      <c r="AJ5" s="46"/>
+      <c r="AK5" s="46"/>
+      <c r="AL5" s="47"/>
+      <c r="AM5" s="45">
         <f>AM6</f>
         <v>45978</v>
       </c>
-      <c r="AN5" s="51"/>
-      <c r="AO5" s="51"/>
-      <c r="AP5" s="51"/>
-      <c r="AQ5" s="51"/>
-      <c r="AR5" s="51"/>
-      <c r="AS5" s="52"/>
-      <c r="AT5" s="50">
+      <c r="AN5" s="46"/>
+      <c r="AO5" s="46"/>
+      <c r="AP5" s="46"/>
+      <c r="AQ5" s="46"/>
+      <c r="AR5" s="46"/>
+      <c r="AS5" s="47"/>
+      <c r="AT5" s="45">
         <f>AT6</f>
         <v>45985</v>
       </c>
-      <c r="AU5" s="51"/>
-      <c r="AV5" s="51"/>
-      <c r="AW5" s="51"/>
-      <c r="AX5" s="51"/>
-      <c r="AY5" s="51"/>
-      <c r="AZ5" s="52"/>
-      <c r="BA5" s="50">
+      <c r="AU5" s="46"/>
+      <c r="AV5" s="46"/>
+      <c r="AW5" s="46"/>
+      <c r="AX5" s="46"/>
+      <c r="AY5" s="46"/>
+      <c r="AZ5" s="47"/>
+      <c r="BA5" s="45">
         <f>BA6</f>
         <v>45992</v>
       </c>
-      <c r="BB5" s="51"/>
-      <c r="BC5" s="51"/>
-      <c r="BD5" s="51"/>
-      <c r="BE5" s="51"/>
-      <c r="BF5" s="51"/>
-      <c r="BG5" s="52"/>
-      <c r="BH5" s="50">
+      <c r="BB5" s="46"/>
+      <c r="BC5" s="46"/>
+      <c r="BD5" s="46"/>
+      <c r="BE5" s="46"/>
+      <c r="BF5" s="46"/>
+      <c r="BG5" s="47"/>
+      <c r="BH5" s="45">
         <f>BH6</f>
         <v>45999</v>
       </c>
-      <c r="BI5" s="51"/>
-      <c r="BJ5" s="51"/>
-      <c r="BK5" s="51"/>
-      <c r="BL5" s="51"/>
-      <c r="BM5" s="51"/>
-      <c r="BN5" s="52"/>
+      <c r="BI5" s="46"/>
+      <c r="BJ5" s="46"/>
+      <c r="BK5" s="46"/>
+      <c r="BL5" s="46"/>
+      <c r="BM5" s="46"/>
+      <c r="BN5" s="47"/>
     </row>
-    <row r="6" spans="1:66" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:66" x14ac:dyDescent="0.4">
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
       <c r="D6" s="6"/>
@@ -2163,271 +2115,269 @@
         <v>46005</v>
       </c>
     </row>
-    <row r="7" spans="1:66" s="2" customFormat="1" ht="23.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="35"/>
+    <row r="7" spans="1:66" s="2" customFormat="1" ht="12.6" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A7" s="34"/>
       <c r="B7" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="52" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="52"/>
+      <c r="E7" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="21" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="E7" s="23" t="s">
+      <c r="F7" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="F7" s="23" t="s">
+      <c r="G7" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="G7" s="21" t="s">
+      <c r="H7" s="21" t="s">
+        <v>8</v>
+      </c>
+      <c r="I7" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="H7" s="21" t="s">
-        <v>9</v>
-      </c>
-      <c r="I7" s="23" t="s">
-        <v>8</v>
-      </c>
       <c r="J7" s="21"/>
-      <c r="K7" s="24" t="str">
+      <c r="K7" s="23" t="str">
         <f t="shared" ref="K7:AP7" si="2">CHOOSE(WEEKDAY(K6,1),"S","M","T","W","T","F","S")</f>
         <v>M</v>
       </c>
-      <c r="L7" s="25" t="str">
+      <c r="L7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>T</v>
       </c>
-      <c r="M7" s="25" t="str">
+      <c r="M7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>W</v>
       </c>
-      <c r="N7" s="25" t="str">
+      <c r="N7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>T</v>
       </c>
-      <c r="O7" s="25" t="str">
+      <c r="O7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>F</v>
       </c>
-      <c r="P7" s="25" t="str">
+      <c r="P7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>S</v>
       </c>
-      <c r="Q7" s="26" t="str">
+      <c r="Q7" s="25" t="str">
         <f t="shared" si="2"/>
         <v>S</v>
       </c>
-      <c r="R7" s="24" t="str">
+      <c r="R7" s="23" t="str">
         <f t="shared" si="2"/>
         <v>M</v>
       </c>
-      <c r="S7" s="25" t="str">
+      <c r="S7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>T</v>
       </c>
-      <c r="T7" s="25" t="str">
+      <c r="T7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>W</v>
       </c>
-      <c r="U7" s="25" t="str">
+      <c r="U7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>T</v>
       </c>
-      <c r="V7" s="25" t="str">
+      <c r="V7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>F</v>
       </c>
-      <c r="W7" s="25" t="str">
+      <c r="W7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>S</v>
       </c>
-      <c r="X7" s="26" t="str">
+      <c r="X7" s="25" t="str">
         <f t="shared" si="2"/>
         <v>S</v>
       </c>
-      <c r="Y7" s="24" t="str">
+      <c r="Y7" s="23" t="str">
         <f t="shared" si="2"/>
         <v>M</v>
       </c>
-      <c r="Z7" s="25" t="str">
+      <c r="Z7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>T</v>
       </c>
-      <c r="AA7" s="25" t="str">
+      <c r="AA7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>W</v>
       </c>
-      <c r="AB7" s="25" t="str">
+      <c r="AB7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>T</v>
       </c>
-      <c r="AC7" s="25" t="str">
+      <c r="AC7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>F</v>
       </c>
-      <c r="AD7" s="25" t="str">
+      <c r="AD7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>S</v>
       </c>
-      <c r="AE7" s="26" t="str">
+      <c r="AE7" s="25" t="str">
         <f t="shared" si="2"/>
         <v>S</v>
       </c>
-      <c r="AF7" s="24" t="str">
+      <c r="AF7" s="23" t="str">
         <f t="shared" si="2"/>
         <v>M</v>
       </c>
-      <c r="AG7" s="25" t="str">
+      <c r="AG7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>T</v>
       </c>
-      <c r="AH7" s="25" t="str">
+      <c r="AH7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>W</v>
       </c>
-      <c r="AI7" s="25" t="str">
+      <c r="AI7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>T</v>
       </c>
-      <c r="AJ7" s="25" t="str">
+      <c r="AJ7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>F</v>
       </c>
-      <c r="AK7" s="25" t="str">
+      <c r="AK7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>S</v>
       </c>
-      <c r="AL7" s="26" t="str">
+      <c r="AL7" s="25" t="str">
         <f t="shared" si="2"/>
         <v>S</v>
       </c>
-      <c r="AM7" s="24" t="str">
+      <c r="AM7" s="23" t="str">
         <f t="shared" si="2"/>
         <v>M</v>
       </c>
-      <c r="AN7" s="25" t="str">
+      <c r="AN7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>T</v>
       </c>
-      <c r="AO7" s="25" t="str">
+      <c r="AO7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>W</v>
       </c>
-      <c r="AP7" s="25" t="str">
+      <c r="AP7" s="24" t="str">
         <f t="shared" si="2"/>
         <v>T</v>
       </c>
-      <c r="AQ7" s="25" t="str">
+      <c r="AQ7" s="24" t="str">
         <f t="shared" ref="AQ7:BN7" si="3">CHOOSE(WEEKDAY(AQ6,1),"S","M","T","W","T","F","S")</f>
         <v>F</v>
       </c>
-      <c r="AR7" s="25" t="str">
+      <c r="AR7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>S</v>
       </c>
-      <c r="AS7" s="26" t="str">
+      <c r="AS7" s="25" t="str">
         <f t="shared" si="3"/>
         <v>S</v>
       </c>
-      <c r="AT7" s="24" t="str">
+      <c r="AT7" s="23" t="str">
         <f t="shared" si="3"/>
         <v>M</v>
       </c>
-      <c r="AU7" s="25" t="str">
+      <c r="AU7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>T</v>
       </c>
-      <c r="AV7" s="25" t="str">
+      <c r="AV7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>W</v>
       </c>
-      <c r="AW7" s="25" t="str">
+      <c r="AW7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>T</v>
       </c>
-      <c r="AX7" s="25" t="str">
+      <c r="AX7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>F</v>
       </c>
-      <c r="AY7" s="25" t="str">
+      <c r="AY7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>S</v>
       </c>
-      <c r="AZ7" s="26" t="str">
+      <c r="AZ7" s="25" t="str">
         <f t="shared" si="3"/>
         <v>S</v>
       </c>
-      <c r="BA7" s="24" t="str">
+      <c r="BA7" s="23" t="str">
         <f t="shared" si="3"/>
         <v>M</v>
       </c>
-      <c r="BB7" s="25" t="str">
+      <c r="BB7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>T</v>
       </c>
-      <c r="BC7" s="25" t="str">
+      <c r="BC7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>W</v>
       </c>
-      <c r="BD7" s="25" t="str">
+      <c r="BD7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>T</v>
       </c>
-      <c r="BE7" s="25" t="str">
+      <c r="BE7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>F</v>
       </c>
-      <c r="BF7" s="25" t="str">
+      <c r="BF7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>S</v>
       </c>
-      <c r="BG7" s="26" t="str">
+      <c r="BG7" s="25" t="str">
         <f t="shared" si="3"/>
         <v>S</v>
       </c>
-      <c r="BH7" s="24" t="str">
+      <c r="BH7" s="23" t="str">
         <f t="shared" si="3"/>
         <v>M</v>
       </c>
-      <c r="BI7" s="25" t="str">
+      <c r="BI7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>T</v>
       </c>
-      <c r="BJ7" s="25" t="str">
+      <c r="BJ7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>W</v>
       </c>
-      <c r="BK7" s="25" t="str">
+      <c r="BK7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>T</v>
       </c>
-      <c r="BL7" s="25" t="str">
+      <c r="BL7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>F</v>
       </c>
-      <c r="BM7" s="25" t="str">
+      <c r="BM7" s="24" t="str">
         <f t="shared" si="3"/>
         <v>S</v>
       </c>
-      <c r="BN7" s="26" t="str">
+      <c r="BN7" s="25" t="str">
         <f t="shared" si="3"/>
         <v>S</v>
       </c>
     </row>
-    <row r="8" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A8" s="36"/>
+    <row r="8" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A8" s="35"/>
       <c r="B8" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D8" s="29"/>
-      <c r="E8" s="37">
+        <v>10</v>
+      </c>
+      <c r="D8" s="28"/>
+      <c r="E8" s="36">
         <v>45919</v>
       </c>
-      <c r="F8" s="38">
+      <c r="F8" s="37">
         <v>45920</v>
       </c>
       <c r="G8" s="10">
@@ -2437,7 +2387,7 @@
         <v>1</v>
       </c>
       <c r="I8" s="12">
-        <f t="shared" ref="I8:I37" si="4">IF(OR(F8=0,E8=0)," - ",NETWORKDAYS(E8,F8))</f>
+        <f t="shared" ref="G8:I39" si="4">IF(OR(F8=0,E8=0)," - ",NETWORKDAYS(E8,F8))</f>
         <v>1</v>
       </c>
       <c r="J8" s="16"/>
@@ -2498,19 +2448,19 @@
       <c r="BM8" s="8"/>
       <c r="BN8" s="8"/>
     </row>
-    <row r="9" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A9" s="36"/>
-      <c r="B9" s="39" t="s">
-        <v>14</v>
+    <row r="9" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A9" s="35"/>
+      <c r="B9" s="38" t="s">
+        <v>13</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D9" s="29"/>
-      <c r="E9" s="37">
+        <v>10</v>
+      </c>
+      <c r="D9" s="28"/>
+      <c r="E9" s="36">
         <v>45919</v>
       </c>
-      <c r="F9" s="38">
+      <c r="F9" s="37">
         <v>45920</v>
       </c>
       <c r="G9" s="10">
@@ -2581,19 +2531,19 @@
       <c r="BM9" s="8"/>
       <c r="BN9" s="8"/>
     </row>
-    <row r="10" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A10" s="36"/>
+    <row r="10" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A10" s="35"/>
       <c r="B10" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D10" s="29"/>
-      <c r="E10" s="37">
+        <v>10</v>
+      </c>
+      <c r="D10" s="28"/>
+      <c r="E10" s="36">
         <v>45919</v>
       </c>
-      <c r="F10" s="38">
+      <c r="F10" s="37">
         <v>45920</v>
       </c>
       <c r="G10" s="10">
@@ -2664,19 +2614,19 @@
       <c r="BM10" s="8"/>
       <c r="BN10" s="8"/>
     </row>
-    <row r="11" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A11" s="36"/>
+    <row r="11" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A11" s="35"/>
       <c r="B11" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11" s="29"/>
-      <c r="E11" s="37">
+        <v>10</v>
+      </c>
+      <c r="D11" s="28"/>
+      <c r="E11" s="36">
         <v>45919</v>
       </c>
-      <c r="F11" s="38">
+      <c r="F11" s="37">
         <v>45922</v>
       </c>
       <c r="G11" s="10">
@@ -2747,19 +2697,19 @@
       <c r="BM11" s="8"/>
       <c r="BN11" s="8"/>
     </row>
-    <row r="12" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A12" s="36"/>
+    <row r="12" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A12" s="35"/>
       <c r="B12" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="29"/>
-      <c r="E12" s="37">
+        <v>10</v>
+      </c>
+      <c r="D12" s="28"/>
+      <c r="E12" s="36">
         <v>45919</v>
       </c>
-      <c r="F12" s="38">
+      <c r="F12" s="37">
         <v>45920</v>
       </c>
       <c r="G12" s="10">
@@ -2830,19 +2780,19 @@
       <c r="BM12" s="8"/>
       <c r="BN12" s="8"/>
     </row>
-    <row r="13" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A13" s="36"/>
+    <row r="13" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A13" s="35"/>
       <c r="B13" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" s="29"/>
-      <c r="E13" s="37">
+        <v>10</v>
+      </c>
+      <c r="D13" s="28"/>
+      <c r="E13" s="36">
         <v>45919</v>
       </c>
-      <c r="F13" s="38">
+      <c r="F13" s="37">
         <v>45920</v>
       </c>
       <c r="G13" s="10">
@@ -2913,19 +2863,19 @@
       <c r="BM13" s="8"/>
       <c r="BN13" s="8"/>
     </row>
-    <row r="14" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A14" s="36"/>
+    <row r="14" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A14" s="35"/>
       <c r="B14" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D14" s="29"/>
-      <c r="E14" s="37">
+        <v>10</v>
+      </c>
+      <c r="D14" s="28"/>
+      <c r="E14" s="36">
         <v>45919</v>
       </c>
-      <c r="F14" s="38">
+      <c r="F14" s="37">
         <v>45920</v>
       </c>
       <c r="G14" s="10">
@@ -2996,19 +2946,19 @@
       <c r="BM14" s="8"/>
       <c r="BN14" s="8"/>
     </row>
-    <row r="15" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A15" s="36"/>
+    <row r="15" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A15" s="35"/>
       <c r="B15" s="9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="29"/>
-      <c r="E15" s="37">
+        <v>10</v>
+      </c>
+      <c r="D15" s="28"/>
+      <c r="E15" s="36">
         <v>45919</v>
       </c>
-      <c r="F15" s="38">
+      <c r="F15" s="37">
         <v>45926</v>
       </c>
       <c r="G15" s="10">
@@ -3079,19 +3029,19 @@
       <c r="BM15" s="8"/>
       <c r="BN15" s="8"/>
     </row>
-    <row r="16" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A16" s="36"/>
+    <row r="16" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A16" s="35"/>
       <c r="B16" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D16" s="29"/>
-      <c r="E16" s="37">
+        <v>10</v>
+      </c>
+      <c r="D16" s="28"/>
+      <c r="E16" s="36">
         <v>45927</v>
       </c>
-      <c r="F16" s="38">
+      <c r="F16" s="37">
         <v>45929</v>
       </c>
       <c r="G16" s="10">
@@ -3162,19 +3112,19 @@
       <c r="BM16" s="8"/>
       <c r="BN16" s="8"/>
     </row>
-    <row r="17" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A17" s="36"/>
-      <c r="B17" s="28" t="s">
-        <v>23</v>
+    <row r="17" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A17" s="35"/>
+      <c r="B17" s="27" t="s">
+        <v>22</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D17" s="29"/>
-      <c r="E17" s="37">
+        <v>10</v>
+      </c>
+      <c r="D17" s="28"/>
+      <c r="E17" s="36">
         <v>45927</v>
       </c>
-      <c r="F17" s="38">
+      <c r="F17" s="37">
         <v>45929</v>
       </c>
       <c r="G17" s="10">
@@ -3245,19 +3195,19 @@
       <c r="BM17" s="8"/>
       <c r="BN17" s="8"/>
     </row>
-    <row r="18" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A18" s="36"/>
-      <c r="B18" s="28" t="s">
-        <v>24</v>
+    <row r="18" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A18" s="35"/>
+      <c r="B18" s="27" t="s">
+        <v>23</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D18" s="29"/>
-      <c r="E18" s="37">
+        <v>10</v>
+      </c>
+      <c r="D18" s="28"/>
+      <c r="E18" s="36">
         <v>45927</v>
       </c>
-      <c r="F18" s="38">
+      <c r="F18" s="37">
         <v>45929</v>
       </c>
       <c r="G18" s="10">
@@ -3328,19 +3278,19 @@
       <c r="BM18" s="8"/>
       <c r="BN18" s="8"/>
     </row>
-    <row r="19" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A19" s="36"/>
-      <c r="B19" s="41" t="s">
-        <v>32</v>
+    <row r="19" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A19" s="35"/>
+      <c r="B19" s="40" t="s">
+        <v>31</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D19" s="29"/>
-      <c r="E19" s="37">
+        <v>10</v>
+      </c>
+      <c r="D19" s="28"/>
+      <c r="E19" s="36">
         <v>45929</v>
       </c>
-      <c r="F19" s="38">
+      <c r="F19" s="37">
         <v>45933</v>
       </c>
       <c r="G19" s="10">
@@ -3411,19 +3361,19 @@
       <c r="BM19" s="8"/>
       <c r="BN19" s="8"/>
     </row>
-    <row r="20" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A20" s="36"/>
-      <c r="B20" s="41" t="s">
-        <v>33</v>
+    <row r="20" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A20" s="35"/>
+      <c r="B20" s="40" t="s">
+        <v>32</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20" s="29"/>
-      <c r="E20" s="37">
+        <v>10</v>
+      </c>
+      <c r="D20" s="28"/>
+      <c r="E20" s="36">
         <v>45929</v>
       </c>
-      <c r="F20" s="38">
+      <c r="F20" s="37">
         <v>45933</v>
       </c>
       <c r="G20" s="10">
@@ -3494,19 +3444,19 @@
       <c r="BM20" s="8"/>
       <c r="BN20" s="8"/>
     </row>
-    <row r="21" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A21" s="36"/>
+    <row r="21" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A21" s="35"/>
       <c r="B21" s="9" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="29"/>
-      <c r="E21" s="37">
+        <v>10</v>
+      </c>
+      <c r="D21" s="28"/>
+      <c r="E21" s="36">
         <v>45929</v>
       </c>
-      <c r="F21" s="38">
+      <c r="F21" s="37">
         <v>45933</v>
       </c>
       <c r="G21" s="10">
@@ -3577,19 +3527,19 @@
       <c r="BM21" s="8"/>
       <c r="BN21" s="8"/>
     </row>
-    <row r="22" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A22" s="36"/>
-      <c r="B22" s="41" t="s">
-        <v>30</v>
+    <row r="22" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A22" s="35"/>
+      <c r="B22" s="40" t="s">
+        <v>29</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D22" s="29"/>
-      <c r="E22" s="37">
+        <v>10</v>
+      </c>
+      <c r="D22" s="28"/>
+      <c r="E22" s="36">
         <v>45929</v>
       </c>
-      <c r="F22" s="38">
+      <c r="F22" s="37">
         <v>45933</v>
       </c>
       <c r="G22" s="10">
@@ -3660,19 +3610,19 @@
       <c r="BM22" s="8"/>
       <c r="BN22" s="8"/>
     </row>
-    <row r="23" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A23" s="36"/>
-      <c r="B23" s="41" t="s">
-        <v>31</v>
+    <row r="23" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A23" s="35"/>
+      <c r="B23" s="40" t="s">
+        <v>30</v>
       </c>
       <c r="C23" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D23" s="29"/>
-      <c r="E23" s="37">
+        <v>10</v>
+      </c>
+      <c r="D23" s="28"/>
+      <c r="E23" s="36">
         <v>45929</v>
       </c>
-      <c r="F23" s="38">
+      <c r="F23" s="37">
         <v>45933</v>
       </c>
       <c r="G23" s="10">
@@ -3743,19 +3693,19 @@
       <c r="BM23" s="8"/>
       <c r="BN23" s="8"/>
     </row>
-    <row r="24" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A24" s="36"/>
-      <c r="B24" s="41" t="s">
-        <v>29</v>
+    <row r="24" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A24" s="35"/>
+      <c r="B24" s="40" t="s">
+        <v>28</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D24" s="29"/>
-      <c r="E24" s="37">
+        <v>10</v>
+      </c>
+      <c r="D24" s="28"/>
+      <c r="E24" s="36">
         <v>45932</v>
       </c>
-      <c r="F24" s="38">
+      <c r="F24" s="37">
         <v>45940</v>
       </c>
       <c r="G24" s="10">
@@ -3826,19 +3776,19 @@
       <c r="BM24" s="8"/>
       <c r="BN24" s="8"/>
     </row>
-    <row r="25" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A25" s="36"/>
-      <c r="B25" s="40" t="s">
-        <v>25</v>
+    <row r="25" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A25" s="35"/>
+      <c r="B25" s="39" t="s">
+        <v>24</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D25" s="29"/>
-      <c r="E25" s="37">
+        <v>10</v>
+      </c>
+      <c r="D25" s="28"/>
+      <c r="E25" s="36">
         <v>45932</v>
       </c>
-      <c r="F25" s="38">
+      <c r="F25" s="37">
         <v>45940</v>
       </c>
       <c r="G25" s="10">
@@ -3909,19 +3859,19 @@
       <c r="BM25" s="8"/>
       <c r="BN25" s="8"/>
     </row>
-    <row r="26" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A26" s="36"/>
-      <c r="B26" s="28" t="s">
-        <v>22</v>
+    <row r="26" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A26" s="35"/>
+      <c r="B26" s="27" t="s">
+        <v>21</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D26" s="29"/>
-      <c r="E26" s="37">
+        <v>10</v>
+      </c>
+      <c r="D26" s="28"/>
+      <c r="E26" s="36">
         <v>45927</v>
       </c>
-      <c r="F26" s="38">
+      <c r="F26" s="37">
         <v>45940</v>
       </c>
       <c r="G26" s="10">
@@ -3992,19 +3942,19 @@
       <c r="BM26" s="8"/>
       <c r="BN26" s="8"/>
     </row>
-    <row r="27" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A27" s="36"/>
-      <c r="B27" s="40" t="s">
-        <v>26</v>
+    <row r="27" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A27" s="35"/>
+      <c r="B27" s="39" t="s">
+        <v>25</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D27" s="29"/>
-      <c r="E27" s="37">
+        <v>10</v>
+      </c>
+      <c r="D27" s="28"/>
+      <c r="E27" s="36">
         <v>45941</v>
       </c>
-      <c r="F27" s="38">
+      <c r="F27" s="37">
         <v>45967</v>
       </c>
       <c r="G27" s="10">
@@ -4075,19 +4025,19 @@
       <c r="BM27" s="8"/>
       <c r="BN27" s="8"/>
     </row>
-    <row r="28" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A28" s="36"/>
-      <c r="B28" s="40" t="s">
-        <v>37</v>
+    <row r="28" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A28" s="35"/>
+      <c r="B28" s="39" t="s">
+        <v>36</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D28" s="29"/>
-      <c r="E28" s="37">
+        <v>10</v>
+      </c>
+      <c r="D28" s="28"/>
+      <c r="E28" s="36">
         <v>45941</v>
       </c>
-      <c r="F28" s="38">
+      <c r="F28" s="37">
         <v>45947</v>
       </c>
       <c r="G28" s="10">
@@ -4158,19 +4108,19 @@
       <c r="BM28" s="8"/>
       <c r="BN28" s="8"/>
     </row>
-    <row r="29" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A29" s="36"/>
-      <c r="B29" s="40" t="s">
-        <v>36</v>
+    <row r="29" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A29" s="35"/>
+      <c r="B29" s="39" t="s">
+        <v>35</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D29" s="29"/>
-      <c r="E29" s="37">
+        <v>10</v>
+      </c>
+      <c r="D29" s="28"/>
+      <c r="E29" s="36">
         <v>45948</v>
       </c>
-      <c r="F29" s="38">
+      <c r="F29" s="37">
         <v>45954</v>
       </c>
       <c r="G29" s="10">
@@ -4241,19 +4191,19 @@
       <c r="BM29" s="8"/>
       <c r="BN29" s="8"/>
     </row>
-    <row r="30" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A30" s="36"/>
-      <c r="B30" s="40" t="s">
-        <v>38</v>
+    <row r="30" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A30" s="35"/>
+      <c r="B30" s="39" t="s">
+        <v>37</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D30" s="29"/>
-      <c r="E30" s="37">
+        <v>10</v>
+      </c>
+      <c r="D30" s="28"/>
+      <c r="E30" s="36">
         <v>45955</v>
       </c>
-      <c r="F30" s="38">
+      <c r="F30" s="37">
         <v>45961</v>
       </c>
       <c r="G30" s="10">
@@ -4324,30 +4274,30 @@
       <c r="BM30" s="8"/>
       <c r="BN30" s="8"/>
     </row>
-    <row r="31" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A31" s="36"/>
-      <c r="B31" s="40" t="s">
+    <row r="31" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A31" s="35"/>
+      <c r="B31" s="39" t="s">
         <v>43</v>
       </c>
       <c r="C31" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D31" s="29"/>
-      <c r="E31" s="37">
-        <v>45962</v>
-      </c>
-      <c r="F31" s="38">
-        <v>45967</v>
+        <v>10</v>
+      </c>
+      <c r="D31" s="28"/>
+      <c r="E31" s="36">
+        <v>45960</v>
+      </c>
+      <c r="F31" s="37">
+        <v>46006</v>
       </c>
       <c r="G31" s="10">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="H31" s="11">
         <v>0</v>
       </c>
       <c r="I31" s="12">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="J31" s="16"/>
       <c r="K31" s="8"/>
@@ -4407,30 +4357,30 @@
       <c r="BM31" s="8"/>
       <c r="BN31" s="8"/>
     </row>
-    <row r="32" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A32" s="36"/>
-      <c r="B32" s="40" t="s">
-        <v>27</v>
+    <row r="32" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A32" s="35"/>
+      <c r="B32" s="39" t="s">
+        <v>42</v>
       </c>
       <c r="C32" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D32" s="29"/>
-      <c r="E32" s="37">
-        <v>45968</v>
-      </c>
-      <c r="F32" s="38">
-        <v>45995</v>
+        <v>10</v>
+      </c>
+      <c r="D32" s="28"/>
+      <c r="E32" s="36">
+        <v>45962</v>
+      </c>
+      <c r="F32" s="37">
+        <v>45967</v>
       </c>
       <c r="G32" s="10">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H32" s="11">
         <v>0</v>
       </c>
       <c r="I32" s="12">
         <f t="shared" si="4"/>
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="J32" s="16"/>
       <c r="K32" s="8"/>
@@ -4490,30 +4440,30 @@
       <c r="BM32" s="8"/>
       <c r="BN32" s="8"/>
     </row>
-    <row r="33" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A33" s="36"/>
-      <c r="B33" s="40" t="s">
-        <v>39</v>
+    <row r="33" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A33" s="35"/>
+      <c r="B33" s="39" t="s">
+        <v>26</v>
       </c>
       <c r="C33" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D33" s="29"/>
-      <c r="E33" s="37">
+        <v>10</v>
+      </c>
+      <c r="D33" s="28"/>
+      <c r="E33" s="36">
         <v>45968</v>
       </c>
-      <c r="F33" s="38">
-        <v>45976</v>
+      <c r="F33" s="37">
+        <v>45995</v>
       </c>
       <c r="G33" s="10">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H33" s="11">
         <v>0</v>
       </c>
       <c r="I33" s="12">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="J33" s="16"/>
       <c r="K33" s="8"/>
@@ -4573,20 +4523,20 @@
       <c r="BM33" s="8"/>
       <c r="BN33" s="8"/>
     </row>
-    <row r="34" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A34" s="36"/>
-      <c r="B34" s="40" t="s">
-        <v>40</v>
+    <row r="34" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A34" s="35"/>
+      <c r="B34" s="39" t="s">
+        <v>38</v>
       </c>
       <c r="C34" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D34" s="29"/>
-      <c r="E34" s="37">
-        <v>45977</v>
-      </c>
-      <c r="F34" s="38">
-        <v>45983</v>
+        <v>10</v>
+      </c>
+      <c r="D34" s="28"/>
+      <c r="E34" s="36">
+        <v>45968</v>
+      </c>
+      <c r="F34" s="37">
+        <v>45976</v>
       </c>
       <c r="G34" s="10">
         <v>1</v>
@@ -4596,7 +4546,7 @@
       </c>
       <c r="I34" s="12">
         <f t="shared" si="4"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J34" s="16"/>
       <c r="K34" s="8"/>
@@ -4656,20 +4606,20 @@
       <c r="BM34" s="8"/>
       <c r="BN34" s="8"/>
     </row>
-    <row r="35" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A35" s="36"/>
-      <c r="B35" s="40" t="s">
-        <v>41</v>
+    <row r="35" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A35" s="35"/>
+      <c r="B35" s="39" t="s">
+        <v>39</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D35" s="29"/>
-      <c r="E35" s="37">
-        <v>45984</v>
-      </c>
-      <c r="F35" s="38">
-        <v>45989</v>
+        <v>10</v>
+      </c>
+      <c r="D35" s="28"/>
+      <c r="E35" s="36">
+        <v>45977</v>
+      </c>
+      <c r="F35" s="37">
+        <v>45983</v>
       </c>
       <c r="G35" s="10">
         <v>1</v>
@@ -4739,30 +4689,30 @@
       <c r="BM35" s="8"/>
       <c r="BN35" s="8"/>
     </row>
-    <row r="36" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A36" s="36"/>
-      <c r="B36" s="40" t="s">
-        <v>42</v>
+    <row r="36" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A36" s="35"/>
+      <c r="B36" s="39" t="s">
+        <v>44</v>
       </c>
       <c r="C36" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D36" s="29"/>
-      <c r="E36" s="37">
-        <v>45990</v>
-      </c>
-      <c r="F36" s="38">
-        <v>45993</v>
+        <v>45</v>
+      </c>
+      <c r="D36" s="28"/>
+      <c r="E36" s="36">
+        <v>45986</v>
+      </c>
+      <c r="F36" s="37">
+        <v>46006</v>
       </c>
       <c r="G36" s="10">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="H36" s="11">
         <v>0</v>
       </c>
       <c r="I36" s="12">
         <f t="shared" si="4"/>
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="J36" s="16"/>
       <c r="K36" s="8"/>
@@ -4822,20 +4772,20 @@
       <c r="BM36" s="8"/>
       <c r="BN36" s="8"/>
     </row>
-    <row r="37" spans="1:66" s="9" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A37" s="36"/>
-      <c r="B37" s="40" t="s">
-        <v>28</v>
+    <row r="37" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A37" s="35"/>
+      <c r="B37" s="39" t="s">
+        <v>40</v>
       </c>
       <c r="C37" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D37" s="29"/>
-      <c r="E37" s="37">
-        <v>45994</v>
-      </c>
-      <c r="F37" s="38">
-        <v>45995</v>
+        <v>10</v>
+      </c>
+      <c r="D37" s="28"/>
+      <c r="E37" s="36">
+        <v>45984</v>
+      </c>
+      <c r="F37" s="37">
+        <v>45989</v>
       </c>
       <c r="G37" s="10">
         <v>1</v>
@@ -4845,7 +4795,7 @@
       </c>
       <c r="I37" s="12">
         <f t="shared" si="4"/>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J37" s="16"/>
       <c r="K37" s="8"/>
@@ -4905,9 +4855,186 @@
       <c r="BM37" s="8"/>
       <c r="BN37" s="8"/>
     </row>
+    <row r="38" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A38" s="35"/>
+      <c r="B38" s="39" t="s">
+        <v>41</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D38" s="28"/>
+      <c r="E38" s="36">
+        <v>45990</v>
+      </c>
+      <c r="F38" s="37">
+        <v>45993</v>
+      </c>
+      <c r="G38" s="10">
+        <v>1</v>
+      </c>
+      <c r="H38" s="11">
+        <v>0</v>
+      </c>
+      <c r="I38" s="12">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="J38" s="16"/>
+      <c r="K38" s="8"/>
+      <c r="L38" s="8"/>
+      <c r="M38" s="8"/>
+      <c r="N38" s="8"/>
+      <c r="O38" s="8"/>
+      <c r="P38" s="8"/>
+      <c r="Q38" s="8"/>
+      <c r="R38" s="8"/>
+      <c r="S38" s="8"/>
+      <c r="T38" s="8"/>
+      <c r="U38" s="8"/>
+      <c r="V38" s="8"/>
+      <c r="W38" s="8"/>
+      <c r="X38" s="8"/>
+      <c r="Y38" s="8"/>
+      <c r="Z38" s="8"/>
+      <c r="AA38" s="8"/>
+      <c r="AB38" s="8"/>
+      <c r="AC38" s="8"/>
+      <c r="AD38" s="8"/>
+      <c r="AE38" s="8"/>
+      <c r="AF38" s="8"/>
+      <c r="AG38" s="8"/>
+      <c r="AH38" s="8"/>
+      <c r="AI38" s="8"/>
+      <c r="AJ38" s="8"/>
+      <c r="AK38" s="8"/>
+      <c r="AL38" s="8"/>
+      <c r="AM38" s="8"/>
+      <c r="AN38" s="8"/>
+      <c r="AO38" s="8"/>
+      <c r="AP38" s="8"/>
+      <c r="AQ38" s="8"/>
+      <c r="AR38" s="8"/>
+      <c r="AS38" s="8"/>
+      <c r="AT38" s="8"/>
+      <c r="AU38" s="8"/>
+      <c r="AV38" s="8"/>
+      <c r="AW38" s="8"/>
+      <c r="AX38" s="8"/>
+      <c r="AY38" s="8"/>
+      <c r="AZ38" s="8"/>
+      <c r="BA38" s="8"/>
+      <c r="BB38" s="8"/>
+      <c r="BC38" s="8"/>
+      <c r="BD38" s="8"/>
+      <c r="BE38" s="8"/>
+      <c r="BF38" s="8"/>
+      <c r="BG38" s="8"/>
+      <c r="BH38" s="8"/>
+      <c r="BI38" s="8"/>
+      <c r="BJ38" s="8"/>
+      <c r="BK38" s="8"/>
+      <c r="BL38" s="8"/>
+      <c r="BM38" s="8"/>
+      <c r="BN38" s="8"/>
+    </row>
+    <row r="39" spans="1:66" s="9" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.4">
+      <c r="A39" s="35"/>
+      <c r="B39" s="39" t="s">
+        <v>27</v>
+      </c>
+      <c r="C39" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D39" s="28"/>
+      <c r="E39" s="36">
+        <v>45994</v>
+      </c>
+      <c r="F39" s="37">
+        <v>45995</v>
+      </c>
+      <c r="G39" s="10">
+        <v>1</v>
+      </c>
+      <c r="H39" s="11">
+        <v>0</v>
+      </c>
+      <c r="I39" s="12">
+        <f t="shared" si="4"/>
+        <v>2</v>
+      </c>
+      <c r="J39" s="16"/>
+      <c r="K39" s="8"/>
+      <c r="L39" s="8"/>
+      <c r="M39" s="8"/>
+      <c r="N39" s="8"/>
+      <c r="O39" s="8"/>
+      <c r="P39" s="8"/>
+      <c r="Q39" s="8"/>
+      <c r="R39" s="8"/>
+      <c r="S39" s="8"/>
+      <c r="T39" s="8"/>
+      <c r="U39" s="8"/>
+      <c r="V39" s="8"/>
+      <c r="W39" s="8"/>
+      <c r="X39" s="8"/>
+      <c r="Y39" s="8"/>
+      <c r="Z39" s="8"/>
+      <c r="AA39" s="8"/>
+      <c r="AB39" s="8"/>
+      <c r="AC39" s="8"/>
+      <c r="AD39" s="8"/>
+      <c r="AE39" s="8"/>
+      <c r="AF39" s="8"/>
+      <c r="AG39" s="8"/>
+      <c r="AH39" s="8"/>
+      <c r="AI39" s="8"/>
+      <c r="AJ39" s="8"/>
+      <c r="AK39" s="8"/>
+      <c r="AL39" s="8"/>
+      <c r="AM39" s="8"/>
+      <c r="AN39" s="8"/>
+      <c r="AO39" s="8"/>
+      <c r="AP39" s="8"/>
+      <c r="AQ39" s="8"/>
+      <c r="AR39" s="8"/>
+      <c r="AS39" s="8"/>
+      <c r="AT39" s="8"/>
+      <c r="AU39" s="8"/>
+      <c r="AV39" s="8"/>
+      <c r="AW39" s="8"/>
+      <c r="AX39" s="8"/>
+      <c r="AY39" s="8"/>
+      <c r="AZ39" s="8"/>
+      <c r="BA39" s="8"/>
+      <c r="BB39" s="8"/>
+      <c r="BC39" s="8"/>
+      <c r="BD39" s="8"/>
+      <c r="BE39" s="8"/>
+      <c r="BF39" s="8"/>
+      <c r="BG39" s="8"/>
+      <c r="BH39" s="8"/>
+      <c r="BI39" s="8"/>
+      <c r="BJ39" s="8"/>
+      <c r="BK39" s="8"/>
+      <c r="BL39" s="8"/>
+      <c r="BM39" s="8"/>
+      <c r="BN39" s="8"/>
+    </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertRows="0" deleteRows="0"/>
-  <mergeCells count="20">
+  <mergeCells count="21">
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="K1:AB1"/>
+    <mergeCell ref="C5:E5"/>
+    <mergeCell ref="R4:X4"/>
+    <mergeCell ref="K4:Q4"/>
+    <mergeCell ref="C4:E4"/>
+    <mergeCell ref="R5:X5"/>
+    <mergeCell ref="K5:Q5"/>
+    <mergeCell ref="Y4:AE4"/>
+    <mergeCell ref="Y5:AE5"/>
     <mergeCell ref="AF4:AL4"/>
     <mergeCell ref="AF5:AL5"/>
     <mergeCell ref="BH4:BN4"/>
@@ -4918,19 +5045,9 @@
     <mergeCell ref="AM4:AS4"/>
     <mergeCell ref="BA4:BG4"/>
     <mergeCell ref="BA5:BG5"/>
-    <mergeCell ref="F4:G4"/>
-    <mergeCell ref="K1:AB1"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="R4:X4"/>
-    <mergeCell ref="K4:Q4"/>
-    <mergeCell ref="C4:E4"/>
-    <mergeCell ref="R5:X5"/>
-    <mergeCell ref="K5:Q5"/>
-    <mergeCell ref="Y4:AE4"/>
-    <mergeCell ref="Y5:AE5"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
-  <conditionalFormatting sqref="H8:H37">
+  <conditionalFormatting sqref="H8:H39">
     <cfRule type="dataBar" priority="10">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -4949,12 +5066,12 @@
       <formula>K$6=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K6:BN37">
+  <conditionalFormatting sqref="K6:BN39">
     <cfRule type="expression" dxfId="2" priority="16">
       <formula>K$6=TODAY()</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K8:BN37">
+  <conditionalFormatting sqref="K8:BN39">
     <cfRule type="expression" dxfId="1" priority="56">
       <formula>AND($E8&lt;=K$6,ROUNDDOWN(($F8-$E8+1)*$H8,0)+$E8-1&gt;=K$6)</formula>
     </cfRule>
@@ -4969,7 +5086,7 @@
   <pageSetup scale="63" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <ignoredErrors>
-    <ignoredError sqref="G12 G11 G17 G10 G9 G33:H36 H28:H31" unlockedFormula="1"/>
+    <ignoredError sqref="G17 G9:G12 G37:H38 H32 H28:H29 G34:H35" unlockedFormula="1"/>
   </ignoredErrors>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
@@ -4985,11 +5102,11 @@
                     <xdr:col>9</xdr:col>
                     <xdr:colOff>95250</xdr:colOff>
                     <xdr:row>1</xdr:row>
-                    <xdr:rowOff>123825</xdr:rowOff>
+                    <xdr:rowOff>125730</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>27</xdr:col>
-                    <xdr:colOff>104775</xdr:colOff>
+                    <xdr:colOff>106680</xdr:colOff>
                     <xdr:row>2</xdr:row>
                     <xdr:rowOff>114300</xdr:rowOff>
                   </to>
@@ -5017,7 +5134,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>H8:H37</xm:sqref>
+          <xm:sqref>H8:H39</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>